<commit_message>
Test modelo final con datos reales
</commit_message>
<xml_diff>
--- a/modelos_tfg/CompletoModelos.xlsx
+++ b/modelos_tfg/CompletoModelos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22C81AB-99A2-4AF9-A0EA-51F2BAC92ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6BEC181-70C4-40D9-BD4B-EDDED2D8A45E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="30" windowWidth="29040" windowHeight="15390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Métricas Validación" sheetId="1" r:id="rId1"/>
@@ -1420,7 +1420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="215">
+  <cellXfs count="214">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -1533,171 +1533,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="19" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="19" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1746,7 +1587,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1768,8 +1609,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1794,12 +1634,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1810,32 +1644,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1852,6 +1668,189 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="14" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1993,7 +1992,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>587377</xdr:colOff>
+      <xdr:colOff>528762</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
@@ -2331,32 +2330,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="105" t="s">
+      <c r="D3" s="188" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="106"/>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="108" t="s">
+      <c r="E3" s="189"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
+      <c r="H3" s="190"/>
+      <c r="I3" s="191" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="109"/>
-      <c r="K3" s="109"/>
-      <c r="L3" s="109"/>
-      <c r="M3" s="109"/>
-      <c r="N3" s="109"/>
-      <c r="O3" s="109"/>
-      <c r="P3" s="109"/>
-      <c r="Q3" s="110"/>
-      <c r="R3" s="115" t="s">
+      <c r="J3" s="192"/>
+      <c r="K3" s="192"/>
+      <c r="L3" s="192"/>
+      <c r="M3" s="192"/>
+      <c r="N3" s="192"/>
+      <c r="O3" s="192"/>
+      <c r="P3" s="192"/>
+      <c r="Q3" s="193"/>
+      <c r="R3" s="198" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="116"/>
-      <c r="T3" s="116"/>
-      <c r="U3" s="116"/>
-      <c r="V3" s="116"/>
-      <c r="W3" s="117"/>
+      <c r="S3" s="199"/>
+      <c r="T3" s="199"/>
+      <c r="U3" s="199"/>
+      <c r="V3" s="199"/>
+      <c r="W3" s="200"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
@@ -2407,16 +2406,16 @@
       <c r="Q4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="118"/>
-      <c r="S4" s="119"/>
-      <c r="T4" s="119"/>
-      <c r="U4" s="119"/>
-      <c r="V4" s="119"/>
-      <c r="W4" s="120"/>
+      <c r="R4" s="201"/>
+      <c r="S4" s="202"/>
+      <c r="T4" s="202"/>
+      <c r="U4" s="202"/>
+      <c r="V4" s="202"/>
+      <c r="W4" s="203"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
-      <c r="B5" s="111" t="s">
+      <c r="B5" s="194" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -2464,18 +2463,18 @@
       <c r="Q5" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="103" t="s">
+      <c r="R5" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="98"/>
-      <c r="T5" s="98"/>
-      <c r="U5" s="98"/>
-      <c r="V5" s="98"/>
-      <c r="W5" s="99"/>
+      <c r="S5" s="181"/>
+      <c r="T5" s="181"/>
+      <c r="U5" s="181"/>
+      <c r="V5" s="181"/>
+      <c r="W5" s="182"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
-      <c r="B6" s="112"/>
+      <c r="B6" s="195"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2521,16 +2520,16 @@
       <c r="Q6" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="91"/>
-      <c r="S6" s="92"/>
-      <c r="T6" s="92"/>
-      <c r="U6" s="92"/>
-      <c r="V6" s="92"/>
-      <c r="W6" s="93"/>
+      <c r="R6" s="174"/>
+      <c r="S6" s="175"/>
+      <c r="T6" s="175"/>
+      <c r="U6" s="175"/>
+      <c r="V6" s="175"/>
+      <c r="W6" s="176"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
-      <c r="B7" s="113"/>
+      <c r="B7" s="196"/>
       <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
@@ -2576,16 +2575,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="94"/>
-      <c r="S7" s="95"/>
-      <c r="T7" s="95"/>
-      <c r="U7" s="95"/>
-      <c r="V7" s="95"/>
-      <c r="W7" s="96"/>
+      <c r="R7" s="177"/>
+      <c r="S7" s="178"/>
+      <c r="T7" s="178"/>
+      <c r="U7" s="178"/>
+      <c r="V7" s="178"/>
+      <c r="W7" s="179"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="114" t="s">
+      <c r="B8" s="197" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -2633,18 +2632,18 @@
       <c r="Q8" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="103" t="s">
+      <c r="R8" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="98"/>
-      <c r="T8" s="98"/>
-      <c r="U8" s="98"/>
-      <c r="V8" s="98"/>
-      <c r="W8" s="99"/>
+      <c r="S8" s="181"/>
+      <c r="T8" s="181"/>
+      <c r="U8" s="181"/>
+      <c r="V8" s="181"/>
+      <c r="W8" s="182"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="112"/>
+      <c r="B9" s="195"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2690,16 +2689,16 @@
       <c r="Q9" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="91"/>
-      <c r="S9" s="92"/>
-      <c r="T9" s="92"/>
-      <c r="U9" s="92"/>
-      <c r="V9" s="92"/>
-      <c r="W9" s="93"/>
+      <c r="R9" s="174"/>
+      <c r="S9" s="175"/>
+      <c r="T9" s="175"/>
+      <c r="U9" s="175"/>
+      <c r="V9" s="175"/>
+      <c r="W9" s="176"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
-      <c r="B10" s="113"/>
+      <c r="B10" s="196"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -2745,15 +2744,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="94"/>
-      <c r="S10" s="95"/>
-      <c r="T10" s="95"/>
-      <c r="U10" s="95"/>
-      <c r="V10" s="95"/>
-      <c r="W10" s="96"/>
+      <c r="R10" s="177"/>
+      <c r="S10" s="178"/>
+      <c r="T10" s="178"/>
+      <c r="U10" s="178"/>
+      <c r="V10" s="178"/>
+      <c r="W10" s="179"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="114" t="s">
+      <c r="B11" s="197" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -2801,17 +2800,17 @@
       <c r="Q11" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="103" t="s">
+      <c r="R11" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="98"/>
-      <c r="T11" s="98"/>
-      <c r="U11" s="98"/>
-      <c r="V11" s="98"/>
-      <c r="W11" s="99"/>
+      <c r="S11" s="181"/>
+      <c r="T11" s="181"/>
+      <c r="U11" s="181"/>
+      <c r="V11" s="181"/>
+      <c r="W11" s="182"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="112"/>
+      <c r="B12" s="195"/>
       <c r="C12" s="25" t="s">
         <v>12</v>
       </c>
@@ -2857,15 +2856,15 @@
       <c r="Q12" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="91"/>
-      <c r="S12" s="92"/>
-      <c r="T12" s="92"/>
-      <c r="U12" s="92"/>
-      <c r="V12" s="92"/>
-      <c r="W12" s="93"/>
+      <c r="R12" s="174"/>
+      <c r="S12" s="175"/>
+      <c r="T12" s="175"/>
+      <c r="U12" s="175"/>
+      <c r="V12" s="175"/>
+      <c r="W12" s="176"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="112"/>
+      <c r="B13" s="195"/>
       <c r="C13" s="26" t="s">
         <v>14</v>
       </c>
@@ -2911,15 +2910,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="94"/>
-      <c r="S13" s="95"/>
-      <c r="T13" s="95"/>
-      <c r="U13" s="95"/>
-      <c r="V13" s="95"/>
-      <c r="W13" s="96"/>
+      <c r="R13" s="177"/>
+      <c r="S13" s="178"/>
+      <c r="T13" s="178"/>
+      <c r="U13" s="178"/>
+      <c r="V13" s="178"/>
+      <c r="W13" s="179"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="114" t="s">
+      <c r="B14" s="197" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="19" t="s">
@@ -2967,17 +2966,17 @@
       <c r="Q14" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="103" t="s">
+      <c r="R14" s="186" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="98"/>
-      <c r="T14" s="98"/>
-      <c r="U14" s="98"/>
-      <c r="V14" s="98"/>
-      <c r="W14" s="99"/>
+      <c r="S14" s="181"/>
+      <c r="T14" s="181"/>
+      <c r="U14" s="181"/>
+      <c r="V14" s="181"/>
+      <c r="W14" s="182"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="112"/>
+      <c r="B15" s="195"/>
       <c r="C15" s="29" t="s">
         <v>12</v>
       </c>
@@ -3023,15 +3022,15 @@
       <c r="Q15" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="91"/>
-      <c r="S15" s="92"/>
-      <c r="T15" s="92"/>
-      <c r="U15" s="92"/>
-      <c r="V15" s="92"/>
-      <c r="W15" s="93"/>
+      <c r="R15" s="174"/>
+      <c r="S15" s="175"/>
+      <c r="T15" s="175"/>
+      <c r="U15" s="175"/>
+      <c r="V15" s="175"/>
+      <c r="W15" s="176"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="113"/>
+      <c r="B16" s="196"/>
       <c r="C16" s="30" t="s">
         <v>14</v>
       </c>
@@ -3077,16 +3076,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="94"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="95"/>
-      <c r="W16" s="96"/>
+      <c r="R16" s="177"/>
+      <c r="S16" s="178"/>
+      <c r="T16" s="178"/>
+      <c r="U16" s="178"/>
+      <c r="V16" s="178"/>
+      <c r="W16" s="179"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
-      <c r="B17" s="117" t="s">
+      <c r="B17" s="200" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="29" t="s">
@@ -3134,18 +3133,18 @@
       <c r="Q17" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="98" t="s">
+      <c r="R17" s="181" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="98"/>
-      <c r="T17" s="98"/>
-      <c r="U17" s="98"/>
-      <c r="V17" s="98"/>
-      <c r="W17" s="99"/>
+      <c r="S17" s="181"/>
+      <c r="T17" s="181"/>
+      <c r="U17" s="181"/>
+      <c r="V17" s="181"/>
+      <c r="W17" s="182"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="121"/>
+      <c r="B18" s="204"/>
       <c r="C18" s="29" t="s">
         <v>12</v>
       </c>
@@ -3191,16 +3190,16 @@
       <c r="Q18" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="92"/>
-      <c r="S18" s="92"/>
-      <c r="T18" s="92"/>
-      <c r="U18" s="92"/>
-      <c r="V18" s="92"/>
-      <c r="W18" s="93"/>
+      <c r="R18" s="175"/>
+      <c r="S18" s="175"/>
+      <c r="T18" s="175"/>
+      <c r="U18" s="175"/>
+      <c r="V18" s="175"/>
+      <c r="W18" s="176"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
-      <c r="B19" s="120"/>
+      <c r="B19" s="203"/>
       <c r="C19" s="30" t="s">
         <v>14</v>
       </c>
@@ -3246,16 +3245,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="95"/>
-      <c r="S19" s="95"/>
-      <c r="T19" s="95"/>
-      <c r="U19" s="95"/>
-      <c r="V19" s="95"/>
-      <c r="W19" s="96"/>
+      <c r="R19" s="178"/>
+      <c r="S19" s="178"/>
+      <c r="T19" s="178"/>
+      <c r="U19" s="178"/>
+      <c r="V19" s="178"/>
+      <c r="W19" s="179"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="114" t="s">
+      <c r="B20" s="197" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="29" t="s">
@@ -3303,18 +3302,18 @@
       <c r="Q20" s="35">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="97" t="s">
+      <c r="R20" s="180" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="98"/>
-      <c r="T20" s="98"/>
-      <c r="U20" s="98"/>
-      <c r="V20" s="98"/>
-      <c r="W20" s="99"/>
+      <c r="S20" s="181"/>
+      <c r="T20" s="181"/>
+      <c r="U20" s="181"/>
+      <c r="V20" s="181"/>
+      <c r="W20" s="182"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="112"/>
+      <c r="B21" s="195"/>
       <c r="C21" s="29" t="s">
         <v>12</v>
       </c>
@@ -3360,16 +3359,16 @@
       <c r="Q21" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="91"/>
-      <c r="S21" s="92"/>
-      <c r="T21" s="92"/>
-      <c r="U21" s="92"/>
-      <c r="V21" s="92"/>
-      <c r="W21" s="93"/>
+      <c r="R21" s="174"/>
+      <c r="S21" s="175"/>
+      <c r="T21" s="175"/>
+      <c r="U21" s="175"/>
+      <c r="V21" s="175"/>
+      <c r="W21" s="176"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
-      <c r="B22" s="113"/>
+      <c r="B22" s="196"/>
       <c r="C22" s="30" t="s">
         <v>14</v>
       </c>
@@ -3415,16 +3414,16 @@
       <c r="Q22" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="94"/>
-      <c r="S22" s="95"/>
-      <c r="T22" s="95"/>
-      <c r="U22" s="95"/>
-      <c r="V22" s="95"/>
-      <c r="W22" s="96"/>
+      <c r="R22" s="177"/>
+      <c r="S22" s="178"/>
+      <c r="T22" s="178"/>
+      <c r="U22" s="178"/>
+      <c r="V22" s="178"/>
+      <c r="W22" s="179"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58"/>
-      <c r="B23" s="86" t="s">
+      <c r="B23" s="169" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="19" t="s">
@@ -3472,18 +3471,18 @@
       <c r="Q23" s="9">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="97" t="s">
+      <c r="R23" s="180" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="98"/>
-      <c r="T23" s="98"/>
-      <c r="U23" s="98"/>
-      <c r="V23" s="98"/>
-      <c r="W23" s="99"/>
+      <c r="S23" s="181"/>
+      <c r="T23" s="181"/>
+      <c r="U23" s="181"/>
+      <c r="V23" s="181"/>
+      <c r="W23" s="182"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="58"/>
-      <c r="B24" s="87"/>
+      <c r="B24" s="170"/>
       <c r="C24" s="29" t="s">
         <v>12</v>
       </c>
@@ -3529,16 +3528,16 @@
       <c r="Q24" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="91"/>
-      <c r="S24" s="92"/>
-      <c r="T24" s="92"/>
-      <c r="U24" s="92"/>
-      <c r="V24" s="92"/>
-      <c r="W24" s="93"/>
+      <c r="R24" s="174"/>
+      <c r="S24" s="175"/>
+      <c r="T24" s="175"/>
+      <c r="U24" s="175"/>
+      <c r="V24" s="175"/>
+      <c r="W24" s="176"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58"/>
-      <c r="B25" s="90"/>
+      <c r="B25" s="173"/>
       <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
@@ -3584,16 +3583,16 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="94"/>
-      <c r="S25" s="95"/>
-      <c r="T25" s="95"/>
-      <c r="U25" s="95"/>
-      <c r="V25" s="95"/>
-      <c r="W25" s="96"/>
+      <c r="R25" s="177"/>
+      <c r="S25" s="178"/>
+      <c r="T25" s="178"/>
+      <c r="U25" s="178"/>
+      <c r="V25" s="178"/>
+      <c r="W25" s="179"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58"/>
-      <c r="B26" s="86" t="s">
+      <c r="B26" s="169" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="19" t="s">
@@ -3641,18 +3640,18 @@
       <c r="Q26" s="35">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="103" t="s">
+      <c r="R26" s="186" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="98"/>
-      <c r="T26" s="98"/>
-      <c r="U26" s="98"/>
-      <c r="V26" s="98"/>
-      <c r="W26" s="99"/>
+      <c r="S26" s="181"/>
+      <c r="T26" s="181"/>
+      <c r="U26" s="181"/>
+      <c r="V26" s="181"/>
+      <c r="W26" s="182"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="58"/>
-      <c r="B27" s="87"/>
+      <c r="B27" s="170"/>
       <c r="C27" s="29" t="s">
         <v>12</v>
       </c>
@@ -3698,16 +3697,16 @@
       <c r="Q27" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="91"/>
-      <c r="S27" s="92"/>
-      <c r="T27" s="92"/>
-      <c r="U27" s="92"/>
-      <c r="V27" s="92"/>
-      <c r="W27" s="93"/>
+      <c r="R27" s="174"/>
+      <c r="S27" s="175"/>
+      <c r="T27" s="175"/>
+      <c r="U27" s="175"/>
+      <c r="V27" s="175"/>
+      <c r="W27" s="176"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="58"/>
-      <c r="B28" s="90"/>
+      <c r="B28" s="173"/>
       <c r="C28" s="30" t="s">
         <v>14</v>
       </c>
@@ -3753,16 +3752,16 @@
       <c r="Q28" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="94"/>
-      <c r="S28" s="95"/>
-      <c r="T28" s="95"/>
-      <c r="U28" s="95"/>
-      <c r="V28" s="95"/>
-      <c r="W28" s="96"/>
+      <c r="R28" s="177"/>
+      <c r="S28" s="178"/>
+      <c r="T28" s="178"/>
+      <c r="U28" s="178"/>
+      <c r="V28" s="178"/>
+      <c r="W28" s="179"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
-      <c r="B29" s="86" t="s">
+      <c r="B29" s="169" t="s">
         <v>34</v>
       </c>
       <c r="C29" s="28" t="s">
@@ -3810,18 +3809,18 @@
       <c r="Q29" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="97" t="s">
+      <c r="R29" s="180" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="98"/>
-      <c r="T29" s="98"/>
-      <c r="U29" s="98"/>
-      <c r="V29" s="98"/>
-      <c r="W29" s="99"/>
+      <c r="S29" s="181"/>
+      <c r="T29" s="181"/>
+      <c r="U29" s="181"/>
+      <c r="V29" s="181"/>
+      <c r="W29" s="182"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="58"/>
-      <c r="B30" s="87"/>
+      <c r="B30" s="170"/>
       <c r="C30" s="25" t="s">
         <v>12</v>
       </c>
@@ -3867,16 +3866,16 @@
       <c r="Q30" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="91"/>
-      <c r="S30" s="92"/>
-      <c r="T30" s="92"/>
-      <c r="U30" s="92"/>
-      <c r="V30" s="92"/>
-      <c r="W30" s="93"/>
+      <c r="R30" s="174"/>
+      <c r="S30" s="175"/>
+      <c r="T30" s="175"/>
+      <c r="U30" s="175"/>
+      <c r="V30" s="175"/>
+      <c r="W30" s="176"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="58"/>
-      <c r="B31" s="90"/>
+      <c r="B31" s="173"/>
       <c r="C31" s="42" t="s">
         <v>14</v>
       </c>
@@ -3922,16 +3921,16 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="94"/>
-      <c r="S31" s="95"/>
-      <c r="T31" s="95"/>
-      <c r="U31" s="95"/>
-      <c r="V31" s="95"/>
-      <c r="W31" s="96"/>
+      <c r="R31" s="177"/>
+      <c r="S31" s="178"/>
+      <c r="T31" s="178"/>
+      <c r="U31" s="178"/>
+      <c r="V31" s="178"/>
+      <c r="W31" s="179"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
-      <c r="B32" s="86" t="s">
+      <c r="B32" s="169" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="28" t="s">
@@ -3979,18 +3978,18 @@
       <c r="Q32" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="103" t="s">
+      <c r="R32" s="186" t="s">
         <v>61</v>
       </c>
-      <c r="S32" s="98"/>
-      <c r="T32" s="98"/>
-      <c r="U32" s="98"/>
-      <c r="V32" s="98"/>
-      <c r="W32" s="99"/>
+      <c r="S32" s="181"/>
+      <c r="T32" s="181"/>
+      <c r="U32" s="181"/>
+      <c r="V32" s="181"/>
+      <c r="W32" s="182"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
-      <c r="B33" s="87"/>
+      <c r="B33" s="170"/>
       <c r="C33" s="25" t="s">
         <v>12</v>
       </c>
@@ -4036,16 +4035,16 @@
       <c r="Q33" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="91"/>
-      <c r="S33" s="92"/>
-      <c r="T33" s="92"/>
-      <c r="U33" s="92"/>
-      <c r="V33" s="92"/>
-      <c r="W33" s="93"/>
+      <c r="R33" s="174"/>
+      <c r="S33" s="175"/>
+      <c r="T33" s="175"/>
+      <c r="U33" s="175"/>
+      <c r="V33" s="175"/>
+      <c r="W33" s="176"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
-      <c r="B34" s="90"/>
+      <c r="B34" s="173"/>
       <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
@@ -4091,16 +4090,16 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="94"/>
-      <c r="S34" s="95"/>
-      <c r="T34" s="95"/>
-      <c r="U34" s="95"/>
-      <c r="V34" s="95"/>
-      <c r="W34" s="96"/>
+      <c r="R34" s="177"/>
+      <c r="S34" s="178"/>
+      <c r="T34" s="178"/>
+      <c r="U34" s="178"/>
+      <c r="V34" s="178"/>
+      <c r="W34" s="179"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="58"/>
-      <c r="B35" s="86" t="s">
+      <c r="B35" s="169" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="25" t="s">
@@ -4148,18 +4147,18 @@
       <c r="Q35" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="97" t="s">
+      <c r="R35" s="180" t="s">
         <v>63</v>
       </c>
-      <c r="S35" s="98"/>
-      <c r="T35" s="98"/>
-      <c r="U35" s="98"/>
-      <c r="V35" s="98"/>
-      <c r="W35" s="99"/>
+      <c r="S35" s="181"/>
+      <c r="T35" s="181"/>
+      <c r="U35" s="181"/>
+      <c r="V35" s="181"/>
+      <c r="W35" s="182"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="58"/>
-      <c r="B36" s="87"/>
+      <c r="B36" s="170"/>
       <c r="C36" s="25" t="s">
         <v>12</v>
       </c>
@@ -4205,16 +4204,16 @@
       <c r="Q36" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="91"/>
-      <c r="S36" s="92"/>
-      <c r="T36" s="92"/>
-      <c r="U36" s="92"/>
-      <c r="V36" s="92"/>
-      <c r="W36" s="93"/>
+      <c r="R36" s="174"/>
+      <c r="S36" s="175"/>
+      <c r="T36" s="175"/>
+      <c r="U36" s="175"/>
+      <c r="V36" s="175"/>
+      <c r="W36" s="176"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="58"/>
-      <c r="B37" s="90"/>
+      <c r="B37" s="173"/>
       <c r="C37" s="30" t="s">
         <v>14</v>
       </c>
@@ -4260,16 +4259,16 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="94"/>
-      <c r="S37" s="95"/>
-      <c r="T37" s="95"/>
-      <c r="U37" s="95"/>
-      <c r="V37" s="95"/>
-      <c r="W37" s="96"/>
+      <c r="R37" s="177"/>
+      <c r="S37" s="178"/>
+      <c r="T37" s="178"/>
+      <c r="U37" s="178"/>
+      <c r="V37" s="178"/>
+      <c r="W37" s="179"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="59"/>
-      <c r="B38" s="86" t="s">
+      <c r="B38" s="169" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="19" t="s">
@@ -4317,16 +4316,16 @@
       <c r="Q38" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="104"/>
-      <c r="S38" s="78"/>
-      <c r="T38" s="78"/>
-      <c r="U38" s="78"/>
-      <c r="V38" s="78"/>
-      <c r="W38" s="79"/>
+      <c r="R38" s="187"/>
+      <c r="S38" s="161"/>
+      <c r="T38" s="161"/>
+      <c r="U38" s="161"/>
+      <c r="V38" s="161"/>
+      <c r="W38" s="162"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="59"/>
-      <c r="B39" s="87"/>
+      <c r="B39" s="170"/>
       <c r="C39" s="29" t="s">
         <v>12</v>
       </c>
@@ -4372,16 +4371,16 @@
       <c r="Q39" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="80"/>
-      <c r="S39" s="81"/>
-      <c r="T39" s="81"/>
-      <c r="U39" s="81"/>
-      <c r="V39" s="81"/>
-      <c r="W39" s="82"/>
+      <c r="R39" s="163"/>
+      <c r="S39" s="164"/>
+      <c r="T39" s="164"/>
+      <c r="U39" s="164"/>
+      <c r="V39" s="164"/>
+      <c r="W39" s="165"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="59"/>
-      <c r="B40" s="90"/>
+      <c r="B40" s="173"/>
       <c r="C40" s="30" t="s">
         <v>14</v>
       </c>
@@ -4427,16 +4426,16 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="100"/>
-      <c r="S40" s="101"/>
-      <c r="T40" s="101"/>
-      <c r="U40" s="101"/>
-      <c r="V40" s="101"/>
-      <c r="W40" s="102"/>
+      <c r="R40" s="183"/>
+      <c r="S40" s="184"/>
+      <c r="T40" s="184"/>
+      <c r="U40" s="184"/>
+      <c r="V40" s="184"/>
+      <c r="W40" s="185"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="59"/>
-      <c r="B41" s="86" t="s">
+      <c r="B41" s="169" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="29" t="s">
@@ -4484,18 +4483,18 @@
       <c r="Q41" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="103" t="s">
+      <c r="R41" s="186" t="s">
         <v>71</v>
       </c>
-      <c r="S41" s="98"/>
-      <c r="T41" s="98"/>
-      <c r="U41" s="98"/>
-      <c r="V41" s="98"/>
-      <c r="W41" s="99"/>
+      <c r="S41" s="181"/>
+      <c r="T41" s="181"/>
+      <c r="U41" s="181"/>
+      <c r="V41" s="181"/>
+      <c r="W41" s="182"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
-      <c r="B42" s="87"/>
+      <c r="B42" s="170"/>
       <c r="C42" s="29" t="s">
         <v>12</v>
       </c>
@@ -4541,16 +4540,16 @@
       <c r="Q42" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="91"/>
-      <c r="S42" s="92"/>
-      <c r="T42" s="92"/>
-      <c r="U42" s="92"/>
-      <c r="V42" s="92"/>
-      <c r="W42" s="93"/>
+      <c r="R42" s="174"/>
+      <c r="S42" s="175"/>
+      <c r="T42" s="175"/>
+      <c r="U42" s="175"/>
+      <c r="V42" s="175"/>
+      <c r="W42" s="176"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="59"/>
-      <c r="B43" s="87"/>
+      <c r="B43" s="170"/>
       <c r="C43" s="29" t="s">
         <v>14</v>
       </c>
@@ -4596,16 +4595,16 @@
       <c r="Q43" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="91"/>
-      <c r="S43" s="92"/>
-      <c r="T43" s="92"/>
-      <c r="U43" s="92"/>
-      <c r="V43" s="92"/>
-      <c r="W43" s="93"/>
+      <c r="R43" s="174"/>
+      <c r="S43" s="175"/>
+      <c r="T43" s="175"/>
+      <c r="U43" s="175"/>
+      <c r="V43" s="175"/>
+      <c r="W43" s="176"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
-      <c r="B44" s="90"/>
+      <c r="B44" s="173"/>
       <c r="C44" s="30" t="s">
         <v>67</v>
       </c>
@@ -4651,16 +4650,16 @@
       <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="94"/>
-      <c r="S44" s="95"/>
-      <c r="T44" s="95"/>
-      <c r="U44" s="95"/>
-      <c r="V44" s="95"/>
-      <c r="W44" s="96"/>
+      <c r="R44" s="177"/>
+      <c r="S44" s="178"/>
+      <c r="T44" s="178"/>
+      <c r="U44" s="178"/>
+      <c r="V44" s="178"/>
+      <c r="W44" s="179"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="59"/>
-      <c r="B45" s="86" t="s">
+      <c r="B45" s="169" t="s">
         <v>55</v>
       </c>
       <c r="C45" s="29" t="s">
@@ -4708,18 +4707,18 @@
       <c r="Q45" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="77" t="s">
+      <c r="R45" s="160" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="78"/>
-      <c r="T45" s="78"/>
-      <c r="U45" s="78"/>
-      <c r="V45" s="78"/>
-      <c r="W45" s="79"/>
+      <c r="S45" s="161"/>
+      <c r="T45" s="161"/>
+      <c r="U45" s="161"/>
+      <c r="V45" s="161"/>
+      <c r="W45" s="162"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="59"/>
-      <c r="B46" s="87"/>
+      <c r="B46" s="170"/>
       <c r="C46" s="29" t="s">
         <v>12</v>
       </c>
@@ -4765,16 +4764,16 @@
       <c r="Q46" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="80"/>
-      <c r="S46" s="81"/>
-      <c r="T46" s="81"/>
-      <c r="U46" s="81"/>
-      <c r="V46" s="81"/>
-      <c r="W46" s="82"/>
+      <c r="R46" s="163"/>
+      <c r="S46" s="164"/>
+      <c r="T46" s="164"/>
+      <c r="U46" s="164"/>
+      <c r="V46" s="164"/>
+      <c r="W46" s="165"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="59"/>
-      <c r="B47" s="87"/>
+      <c r="B47" s="170"/>
       <c r="C47" s="29" t="s">
         <v>14</v>
       </c>
@@ -4820,16 +4819,16 @@
       <c r="Q47" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="80"/>
-      <c r="S47" s="81"/>
-      <c r="T47" s="81"/>
-      <c r="U47" s="81"/>
-      <c r="V47" s="81"/>
-      <c r="W47" s="82"/>
+      <c r="R47" s="163"/>
+      <c r="S47" s="164"/>
+      <c r="T47" s="164"/>
+      <c r="U47" s="164"/>
+      <c r="V47" s="164"/>
+      <c r="W47" s="165"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
-      <c r="B48" s="90"/>
+      <c r="B48" s="173"/>
       <c r="C48" s="30" t="s">
         <v>67</v>
       </c>
@@ -4875,16 +4874,16 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="100"/>
-      <c r="S48" s="101"/>
-      <c r="T48" s="101"/>
-      <c r="U48" s="101"/>
-      <c r="V48" s="101"/>
-      <c r="W48" s="102"/>
+      <c r="R48" s="183"/>
+      <c r="S48" s="184"/>
+      <c r="T48" s="184"/>
+      <c r="U48" s="184"/>
+      <c r="V48" s="184"/>
+      <c r="W48" s="185"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58"/>
-      <c r="B49" s="86" t="s">
+      <c r="B49" s="169" t="s">
         <v>58</v>
       </c>
       <c r="C49" s="29" t="s">
@@ -4932,18 +4931,18 @@
       <c r="Q49" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="97" t="s">
+      <c r="R49" s="180" t="s">
         <v>79</v>
       </c>
-      <c r="S49" s="98"/>
-      <c r="T49" s="98"/>
-      <c r="U49" s="98"/>
-      <c r="V49" s="98"/>
-      <c r="W49" s="99"/>
+      <c r="S49" s="181"/>
+      <c r="T49" s="181"/>
+      <c r="U49" s="181"/>
+      <c r="V49" s="181"/>
+      <c r="W49" s="182"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="58"/>
-      <c r="B50" s="87"/>
+      <c r="B50" s="170"/>
       <c r="C50" s="29" t="s">
         <v>12</v>
       </c>
@@ -4989,16 +4988,16 @@
       <c r="Q50" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="91"/>
-      <c r="S50" s="92"/>
-      <c r="T50" s="92"/>
-      <c r="U50" s="92"/>
-      <c r="V50" s="92"/>
-      <c r="W50" s="93"/>
+      <c r="R50" s="174"/>
+      <c r="S50" s="175"/>
+      <c r="T50" s="175"/>
+      <c r="U50" s="175"/>
+      <c r="V50" s="175"/>
+      <c r="W50" s="176"/>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="58"/>
-      <c r="B51" s="87"/>
+      <c r="B51" s="170"/>
       <c r="C51" s="29" t="s">
         <v>14</v>
       </c>
@@ -5044,16 +5043,16 @@
       <c r="Q51" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="91"/>
-      <c r="S51" s="92"/>
-      <c r="T51" s="92"/>
-      <c r="U51" s="92"/>
-      <c r="V51" s="92"/>
-      <c r="W51" s="93"/>
+      <c r="R51" s="174"/>
+      <c r="S51" s="175"/>
+      <c r="T51" s="175"/>
+      <c r="U51" s="175"/>
+      <c r="V51" s="175"/>
+      <c r="W51" s="176"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="58"/>
-      <c r="B52" s="90"/>
+      <c r="B52" s="173"/>
       <c r="C52" s="30" t="s">
         <v>67</v>
       </c>
@@ -5099,16 +5098,16 @@
       <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="94"/>
-      <c r="S52" s="95"/>
-      <c r="T52" s="95"/>
-      <c r="U52" s="95"/>
-      <c r="V52" s="95"/>
-      <c r="W52" s="96"/>
+      <c r="R52" s="177"/>
+      <c r="S52" s="178"/>
+      <c r="T52" s="178"/>
+      <c r="U52" s="178"/>
+      <c r="V52" s="178"/>
+      <c r="W52" s="179"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="59"/>
-      <c r="B53" s="86" t="s">
+      <c r="B53" s="169" t="s">
         <v>77</v>
       </c>
       <c r="C53" s="19" t="s">
@@ -5156,18 +5155,18 @@
       <c r="Q53" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="97" t="s">
+      <c r="R53" s="180" t="s">
         <v>80</v>
       </c>
-      <c r="S53" s="98"/>
-      <c r="T53" s="98"/>
-      <c r="U53" s="98"/>
-      <c r="V53" s="98"/>
-      <c r="W53" s="99"/>
+      <c r="S53" s="181"/>
+      <c r="T53" s="181"/>
+      <c r="U53" s="181"/>
+      <c r="V53" s="181"/>
+      <c r="W53" s="182"/>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="59"/>
-      <c r="B54" s="87"/>
+      <c r="B54" s="170"/>
       <c r="C54" s="29" t="s">
         <v>12</v>
       </c>
@@ -5213,16 +5212,16 @@
       <c r="Q54" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R54" s="91"/>
-      <c r="S54" s="92"/>
-      <c r="T54" s="92"/>
-      <c r="U54" s="92"/>
-      <c r="V54" s="92"/>
-      <c r="W54" s="93"/>
+      <c r="R54" s="174"/>
+      <c r="S54" s="175"/>
+      <c r="T54" s="175"/>
+      <c r="U54" s="175"/>
+      <c r="V54" s="175"/>
+      <c r="W54" s="176"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="59"/>
-      <c r="B55" s="87"/>
+      <c r="B55" s="170"/>
       <c r="C55" s="29" t="s">
         <v>14</v>
       </c>
@@ -5268,16 +5267,16 @@
       <c r="Q55" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R55" s="91"/>
-      <c r="S55" s="92"/>
-      <c r="T55" s="92"/>
-      <c r="U55" s="92"/>
-      <c r="V55" s="92"/>
-      <c r="W55" s="93"/>
+      <c r="R55" s="174"/>
+      <c r="S55" s="175"/>
+      <c r="T55" s="175"/>
+      <c r="U55" s="175"/>
+      <c r="V55" s="175"/>
+      <c r="W55" s="176"/>
     </row>
     <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="59"/>
-      <c r="B56" s="90"/>
+      <c r="B56" s="173"/>
       <c r="C56" s="30" t="s">
         <v>67</v>
       </c>
@@ -5323,16 +5322,16 @@
       <c r="Q56" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R56" s="94"/>
-      <c r="S56" s="95"/>
-      <c r="T56" s="95"/>
-      <c r="U56" s="95"/>
-      <c r="V56" s="95"/>
-      <c r="W56" s="96"/>
+      <c r="R56" s="177"/>
+      <c r="S56" s="178"/>
+      <c r="T56" s="178"/>
+      <c r="U56" s="178"/>
+      <c r="V56" s="178"/>
+      <c r="W56" s="179"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
-      <c r="B57" s="86" t="s">
+      <c r="B57" s="169" t="s">
         <v>81</v>
       </c>
       <c r="C57" s="19" t="s">
@@ -5380,18 +5379,18 @@
       <c r="Q57" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="97" t="s">
+      <c r="R57" s="180" t="s">
         <v>87</v>
       </c>
-      <c r="S57" s="98"/>
-      <c r="T57" s="98"/>
-      <c r="U57" s="98"/>
-      <c r="V57" s="98"/>
-      <c r="W57" s="99"/>
+      <c r="S57" s="181"/>
+      <c r="T57" s="181"/>
+      <c r="U57" s="181"/>
+      <c r="V57" s="181"/>
+      <c r="W57" s="182"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="58"/>
-      <c r="B58" s="87"/>
+      <c r="B58" s="170"/>
       <c r="C58" s="29" t="s">
         <v>12</v>
       </c>
@@ -5437,16 +5436,16 @@
       <c r="Q58" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R58" s="91"/>
-      <c r="S58" s="92"/>
-      <c r="T58" s="92"/>
-      <c r="U58" s="92"/>
-      <c r="V58" s="92"/>
-      <c r="W58" s="93"/>
+      <c r="R58" s="174"/>
+      <c r="S58" s="175"/>
+      <c r="T58" s="175"/>
+      <c r="U58" s="175"/>
+      <c r="V58" s="175"/>
+      <c r="W58" s="176"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
-      <c r="B59" s="87"/>
+      <c r="B59" s="170"/>
       <c r="C59" s="29" t="s">
         <v>14</v>
       </c>
@@ -5492,16 +5491,16 @@
       <c r="Q59" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R59" s="91"/>
-      <c r="S59" s="92"/>
-      <c r="T59" s="92"/>
-      <c r="U59" s="92"/>
-      <c r="V59" s="92"/>
-      <c r="W59" s="93"/>
+      <c r="R59" s="174"/>
+      <c r="S59" s="175"/>
+      <c r="T59" s="175"/>
+      <c r="U59" s="175"/>
+      <c r="V59" s="175"/>
+      <c r="W59" s="176"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="58"/>
-      <c r="B60" s="90"/>
+      <c r="B60" s="173"/>
       <c r="C60" s="30" t="s">
         <v>67</v>
       </c>
@@ -5547,16 +5546,16 @@
       <c r="Q60" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R60" s="94"/>
-      <c r="S60" s="95"/>
-      <c r="T60" s="95"/>
-      <c r="U60" s="95"/>
-      <c r="V60" s="95"/>
-      <c r="W60" s="96"/>
+      <c r="R60" s="177"/>
+      <c r="S60" s="178"/>
+      <c r="T60" s="178"/>
+      <c r="U60" s="178"/>
+      <c r="V60" s="178"/>
+      <c r="W60" s="179"/>
     </row>
     <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="86" t="s">
+      <c r="B61" s="169" t="s">
         <v>84</v>
       </c>
       <c r="C61" s="28" t="s">
@@ -5604,18 +5603,18 @@
       <c r="Q61" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R61" s="77" t="s">
+      <c r="R61" s="160" t="s">
         <v>85</v>
       </c>
-      <c r="S61" s="78"/>
-      <c r="T61" s="78"/>
-      <c r="U61" s="78"/>
-      <c r="V61" s="78"/>
-      <c r="W61" s="79"/>
+      <c r="S61" s="161"/>
+      <c r="T61" s="161"/>
+      <c r="U61" s="161"/>
+      <c r="V61" s="161"/>
+      <c r="W61" s="162"/>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="87"/>
+      <c r="B62" s="170"/>
       <c r="C62" s="25" t="s">
         <v>12</v>
       </c>
@@ -5661,16 +5660,16 @@
       <c r="Q62" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R62" s="80"/>
-      <c r="S62" s="81"/>
-      <c r="T62" s="81"/>
-      <c r="U62" s="81"/>
-      <c r="V62" s="81"/>
-      <c r="W62" s="82"/>
+      <c r="R62" s="163"/>
+      <c r="S62" s="164"/>
+      <c r="T62" s="164"/>
+      <c r="U62" s="164"/>
+      <c r="V62" s="164"/>
+      <c r="W62" s="165"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="87"/>
+      <c r="B63" s="170"/>
       <c r="C63" s="25" t="s">
         <v>14</v>
       </c>
@@ -5716,16 +5715,16 @@
       <c r="Q63" s="64">
         <v>1E-3</v>
       </c>
-      <c r="R63" s="80"/>
-      <c r="S63" s="81"/>
-      <c r="T63" s="81"/>
-      <c r="U63" s="81"/>
-      <c r="V63" s="81"/>
-      <c r="W63" s="82"/>
+      <c r="R63" s="163"/>
+      <c r="S63" s="164"/>
+      <c r="T63" s="164"/>
+      <c r="U63" s="164"/>
+      <c r="V63" s="164"/>
+      <c r="W63" s="165"/>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="87"/>
+      <c r="B64" s="170"/>
       <c r="C64" s="25" t="s">
         <v>67</v>
       </c>
@@ -5771,16 +5770,16 @@
       <c r="Q64" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R64" s="80"/>
-      <c r="S64" s="81"/>
-      <c r="T64" s="81"/>
-      <c r="U64" s="81"/>
-      <c r="V64" s="81"/>
-      <c r="W64" s="82"/>
+      <c r="R64" s="163"/>
+      <c r="S64" s="164"/>
+      <c r="T64" s="164"/>
+      <c r="U64" s="164"/>
+      <c r="V64" s="164"/>
+      <c r="W64" s="165"/>
     </row>
     <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="7"/>
-      <c r="B65" s="90"/>
+      <c r="B65" s="173"/>
       <c r="C65" s="67" t="s">
         <v>83</v>
       </c>
@@ -5826,15 +5825,15 @@
       <c r="Q65" s="69">
         <v>1E-3</v>
       </c>
-      <c r="R65" s="100"/>
-      <c r="S65" s="101"/>
-      <c r="T65" s="101"/>
-      <c r="U65" s="101"/>
-      <c r="V65" s="101"/>
-      <c r="W65" s="102"/>
+      <c r="R65" s="183"/>
+      <c r="S65" s="184"/>
+      <c r="T65" s="184"/>
+      <c r="U65" s="184"/>
+      <c r="V65" s="184"/>
+      <c r="W65" s="185"/>
     </row>
     <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="86" t="s">
+      <c r="B66" s="169" t="s">
         <v>86</v>
       </c>
       <c r="C66" s="19" t="s">
@@ -5882,17 +5881,17 @@
       <c r="Q66" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R66" s="77" t="s">
+      <c r="R66" s="160" t="s">
         <v>88</v>
       </c>
-      <c r="S66" s="78"/>
-      <c r="T66" s="78"/>
-      <c r="U66" s="78"/>
-      <c r="V66" s="78"/>
-      <c r="W66" s="79"/>
+      <c r="S66" s="161"/>
+      <c r="T66" s="161"/>
+      <c r="U66" s="161"/>
+      <c r="V66" s="161"/>
+      <c r="W66" s="162"/>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B67" s="87"/>
+      <c r="B67" s="170"/>
       <c r="C67" s="29" t="s">
         <v>12</v>
       </c>
@@ -5938,15 +5937,15 @@
       <c r="Q67" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R67" s="80"/>
-      <c r="S67" s="81"/>
-      <c r="T67" s="81"/>
-      <c r="U67" s="81"/>
-      <c r="V67" s="81"/>
-      <c r="W67" s="82"/>
+      <c r="R67" s="163"/>
+      <c r="S67" s="164"/>
+      <c r="T67" s="164"/>
+      <c r="U67" s="164"/>
+      <c r="V67" s="164"/>
+      <c r="W67" s="165"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B68" s="87"/>
+      <c r="B68" s="170"/>
       <c r="C68" s="29" t="s">
         <v>14</v>
       </c>
@@ -5992,15 +5991,15 @@
       <c r="Q68" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R68" s="80"/>
-      <c r="S68" s="81"/>
-      <c r="T68" s="81"/>
-      <c r="U68" s="81"/>
-      <c r="V68" s="81"/>
-      <c r="W68" s="82"/>
+      <c r="R68" s="163"/>
+      <c r="S68" s="164"/>
+      <c r="T68" s="164"/>
+      <c r="U68" s="164"/>
+      <c r="V68" s="164"/>
+      <c r="W68" s="165"/>
     </row>
     <row r="69" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="88"/>
+      <c r="B69" s="171"/>
       <c r="C69" s="29" t="s">
         <v>67</v>
       </c>
@@ -6046,15 +6045,15 @@
       <c r="Q69" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R69" s="83"/>
-      <c r="S69" s="84"/>
-      <c r="T69" s="84"/>
-      <c r="U69" s="84"/>
-      <c r="V69" s="84"/>
-      <c r="W69" s="85"/>
+      <c r="R69" s="166"/>
+      <c r="S69" s="167"/>
+      <c r="T69" s="167"/>
+      <c r="U69" s="167"/>
+      <c r="V69" s="167"/>
+      <c r="W69" s="168"/>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B70" s="89" t="s">
+      <c r="B70" s="172" t="s">
         <v>89</v>
       </c>
       <c r="C70" s="72" t="s">
@@ -6102,17 +6101,17 @@
       <c r="Q70" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R70" s="91" t="s">
+      <c r="R70" s="174" t="s">
         <v>90</v>
       </c>
-      <c r="S70" s="92"/>
-      <c r="T70" s="92"/>
-      <c r="U70" s="92"/>
-      <c r="V70" s="92"/>
-      <c r="W70" s="93"/>
+      <c r="S70" s="175"/>
+      <c r="T70" s="175"/>
+      <c r="U70" s="175"/>
+      <c r="V70" s="175"/>
+      <c r="W70" s="176"/>
     </row>
     <row r="71" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B71" s="87"/>
+      <c r="B71" s="170"/>
       <c r="C71" s="29" t="s">
         <v>12</v>
       </c>
@@ -6158,15 +6157,15 @@
       <c r="Q71" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R71" s="91"/>
-      <c r="S71" s="92"/>
-      <c r="T71" s="92"/>
-      <c r="U71" s="92"/>
-      <c r="V71" s="92"/>
-      <c r="W71" s="93"/>
+      <c r="R71" s="174"/>
+      <c r="S71" s="175"/>
+      <c r="T71" s="175"/>
+      <c r="U71" s="175"/>
+      <c r="V71" s="175"/>
+      <c r="W71" s="176"/>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B72" s="87"/>
+      <c r="B72" s="170"/>
       <c r="C72" s="29" t="s">
         <v>14</v>
       </c>
@@ -6212,15 +6211,15 @@
       <c r="Q72" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R72" s="91"/>
-      <c r="S72" s="92"/>
-      <c r="T72" s="92"/>
-      <c r="U72" s="92"/>
-      <c r="V72" s="92"/>
-      <c r="W72" s="93"/>
+      <c r="R72" s="174"/>
+      <c r="S72" s="175"/>
+      <c r="T72" s="175"/>
+      <c r="U72" s="175"/>
+      <c r="V72" s="175"/>
+      <c r="W72" s="176"/>
     </row>
     <row r="73" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="90"/>
+      <c r="B73" s="173"/>
       <c r="C73" s="30" t="s">
         <v>67</v>
       </c>
@@ -6266,12 +6265,12 @@
       <c r="Q73" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R73" s="94"/>
-      <c r="S73" s="95"/>
-      <c r="T73" s="95"/>
-      <c r="U73" s="95"/>
-      <c r="V73" s="95"/>
-      <c r="W73" s="96"/>
+      <c r="R73" s="177"/>
+      <c r="S73" s="178"/>
+      <c r="T73" s="178"/>
+      <c r="U73" s="178"/>
+      <c r="V73" s="178"/>
+      <c r="W73" s="179"/>
     </row>
     <row r="74" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -6332,531 +6331,513 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="207" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
+      <c r="C2" s="207"/>
+      <c r="D2" s="207"/>
+      <c r="E2" s="207"/>
+      <c r="F2" s="207"/>
+      <c r="G2" s="207"/>
+      <c r="H2" s="207"/>
+      <c r="I2" s="207"/>
+      <c r="J2" s="207"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="169"/>
-      <c r="C4" s="170"/>
-      <c r="D4" s="187" t="s">
+      <c r="C4" s="116"/>
+      <c r="D4" s="131" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="187" t="s">
+      <c r="E4" s="131" t="s">
         <v>92</v>
       </c>
-      <c r="F4" s="187" t="s">
+      <c r="F4" s="131" t="s">
         <v>93</v>
       </c>
-      <c r="G4" s="187" t="s">
+      <c r="G4" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="187" t="s">
+      <c r="H4" s="131" t="s">
         <v>94</v>
       </c>
-      <c r="I4" s="188" t="s">
+      <c r="I4" s="132" t="s">
         <v>95</v>
       </c>
-      <c r="J4" s="169"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="189" t="s">
+      <c r="B5" s="211" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="190" t="s">
+      <c r="C5" s="133" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="191">
+      <c r="D5" s="134">
         <v>51.7</v>
       </c>
-      <c r="E5" s="192">
+      <c r="E5" s="135">
         <v>118.3</v>
       </c>
-      <c r="F5" s="192">
+      <c r="F5" s="135">
         <v>92.9</v>
       </c>
-      <c r="G5" s="192">
+      <c r="G5" s="135">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H5" s="192">
+      <c r="H5" s="135">
         <v>0.80200000000000005</v>
       </c>
-      <c r="I5" s="191">
+      <c r="I5" s="134">
         <v>31.8</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="193"/>
-      <c r="C6" s="194" t="s">
+      <c r="B6" s="212"/>
+      <c r="C6" s="136" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="141">
+      <c r="D6" s="88">
         <v>51.8</v>
       </c>
-      <c r="E6" s="176">
+      <c r="E6" s="122">
         <v>118.4</v>
       </c>
-      <c r="F6" s="176">
+      <c r="F6" s="122">
         <v>93</v>
       </c>
-      <c r="G6" s="176">
+      <c r="G6" s="122">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H6" s="176">
+      <c r="H6" s="122">
         <v>0.80210000000000004</v>
       </c>
-      <c r="I6" s="141">
+      <c r="I6" s="88">
         <v>19.899999999999999</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="195" t="s">
+      <c r="B7" s="213" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="171" t="s">
+      <c r="C7" s="117" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="139">
+      <c r="D7" s="86">
         <v>48.1</v>
       </c>
-      <c r="E7" s="172">
+      <c r="E7" s="118">
         <v>125.7</v>
       </c>
-      <c r="F7" s="172">
+      <c r="F7" s="118">
         <v>102.5</v>
       </c>
-      <c r="G7" s="172">
+      <c r="G7" s="118">
         <v>0.93859999999999999</v>
       </c>
-      <c r="H7" s="172">
+      <c r="H7" s="118">
         <v>0.755</v>
       </c>
-      <c r="I7" s="139">
+      <c r="I7" s="86">
         <v>27.7</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="193"/>
-      <c r="C8" s="194" t="s">
+      <c r="B8" s="212"/>
+      <c r="C8" s="136" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="141">
+      <c r="D8" s="88">
         <v>48.1</v>
       </c>
-      <c r="E8" s="176">
+      <c r="E8" s="122">
         <v>125.6</v>
       </c>
-      <c r="F8" s="176">
+      <c r="F8" s="122">
         <v>102.4</v>
       </c>
-      <c r="G8" s="176">
+      <c r="G8" s="122">
         <v>0.93869999999999998</v>
       </c>
-      <c r="H8" s="176">
+      <c r="H8" s="122">
         <v>0.75539999999999996</v>
       </c>
-      <c r="I8" s="141">
+      <c r="I8" s="88">
         <v>19.8</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="178"/>
-      <c r="C10" s="207" t="s">
+      <c r="B10" s="124"/>
+      <c r="C10" s="145" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="206" t="s">
+      <c r="D10" s="144" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="144" t="s">
+      <c r="B11" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="208">
+      <c r="C11" s="146">
         <v>0.1</v>
       </c>
-      <c r="D11" s="209">
+      <c r="D11" s="147">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="144" t="s">
+      <c r="B12" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="210">
+      <c r="C12" s="148">
         <v>0</v>
       </c>
-      <c r="D12" s="211">
+      <c r="D12" s="149">
         <v>-1E-4</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="207" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="76"/>
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
-      <c r="F14" s="76"/>
-      <c r="G14" s="76"/>
-      <c r="H14" s="76"/>
-      <c r="I14" s="76"/>
-      <c r="J14" s="76"/>
+      <c r="C14" s="207"/>
+      <c r="D14" s="207"/>
+      <c r="E14" s="207"/>
+      <c r="F14" s="207"/>
+      <c r="G14" s="207"/>
+      <c r="H14" s="207"/>
+      <c r="I14" s="207"/>
+      <c r="J14" s="207"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D15" s="178"/>
-      <c r="E15" s="178"/>
-      <c r="F15" s="178"/>
-      <c r="G15" s="178"/>
-      <c r="H15" s="178"/>
-      <c r="I15" s="178"/>
+      <c r="D15" s="124"/>
+      <c r="E15" s="124"/>
+      <c r="F15" s="124"/>
+      <c r="G15" s="124"/>
+      <c r="H15" s="124"/>
+      <c r="I15" s="124"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="178"/>
-      <c r="C16" s="179"/>
-      <c r="D16" s="182" t="s">
+      <c r="B16" s="124"/>
+      <c r="C16" s="125"/>
+      <c r="D16" s="128" t="s">
         <v>91</v>
       </c>
-      <c r="E16" s="181" t="s">
+      <c r="E16" s="127" t="s">
         <v>92</v>
       </c>
-      <c r="F16" s="180" t="s">
+      <c r="F16" s="126" t="s">
         <v>93</v>
       </c>
-      <c r="G16" s="181" t="s">
+      <c r="G16" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="H16" s="181" t="s">
+      <c r="H16" s="127" t="s">
         <v>94</v>
       </c>
-      <c r="I16" s="182" t="s">
+      <c r="I16" s="128" t="s">
         <v>95</v>
       </c>
-      <c r="J16" s="169"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="185"/>
-      <c r="B17" s="183" t="s">
+      <c r="A17" s="129"/>
+      <c r="B17" s="205" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="177" t="s">
+      <c r="C17" s="123" t="s">
         <v>96</v>
       </c>
-      <c r="D17" s="139">
+      <c r="D17" s="86">
         <v>51.7</v>
       </c>
-      <c r="E17" s="172">
+      <c r="E17" s="118">
         <v>118.3</v>
       </c>
-      <c r="F17" s="172">
+      <c r="F17" s="118">
         <v>92.9</v>
       </c>
-      <c r="G17" s="172">
+      <c r="G17" s="118">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H17" s="172">
+      <c r="H17" s="118">
         <v>0.80200000000000005</v>
       </c>
-      <c r="I17" s="172">
+      <c r="I17" s="118">
         <v>73.400000000000006</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="185"/>
-      <c r="B18" s="184"/>
-      <c r="C18" s="175" t="s">
+      <c r="A18" s="129"/>
+      <c r="B18" s="206"/>
+      <c r="C18" s="121" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="141">
+      <c r="D18" s="88">
         <v>51.7</v>
       </c>
-      <c r="E18" s="176">
+      <c r="E18" s="122">
         <v>128.1</v>
       </c>
-      <c r="F18" s="176">
+      <c r="F18" s="122">
         <v>101.5</v>
       </c>
-      <c r="G18" s="176">
+      <c r="G18" s="122">
         <v>0.93969999999999998</v>
       </c>
-      <c r="H18" s="176">
+      <c r="H18" s="122">
         <v>0.76419999999999999</v>
       </c>
-      <c r="I18" s="176">
+      <c r="I18" s="122">
         <v>88.6</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="185"/>
-      <c r="B19" s="183" t="s">
+      <c r="A19" s="129"/>
+      <c r="B19" s="205" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="173" t="s">
+      <c r="C19" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="139">
+      <c r="D19" s="86">
         <v>48.1</v>
       </c>
-      <c r="E19" s="172">
+      <c r="E19" s="118">
         <v>125.7</v>
       </c>
-      <c r="F19" s="172">
+      <c r="F19" s="118">
         <v>102.5</v>
       </c>
-      <c r="G19" s="172">
+      <c r="G19" s="118">
         <v>0.93859999999999999</v>
       </c>
-      <c r="H19" s="172">
+      <c r="H19" s="118">
         <v>0.755</v>
       </c>
-      <c r="I19" s="172">
+      <c r="I19" s="118">
         <v>79.099999999999994</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="185"/>
-      <c r="B20" s="184"/>
-      <c r="C20" s="175" t="s">
+      <c r="A20" s="129"/>
+      <c r="B20" s="206"/>
+      <c r="C20" s="121" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="141">
+      <c r="D20" s="88">
         <v>53.9</v>
       </c>
-      <c r="E20" s="176">
+      <c r="E20" s="122">
         <v>138.80000000000001</v>
       </c>
-      <c r="F20" s="176">
+      <c r="F20" s="122">
         <v>111.4</v>
       </c>
-      <c r="G20" s="176">
+      <c r="G20" s="122">
         <v>0.9274</v>
       </c>
-      <c r="H20" s="176">
+      <c r="H20" s="122">
         <v>0.71409999999999996</v>
       </c>
-      <c r="I20" s="176">
+      <c r="I20" s="122">
         <v>149.80000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="169"/>
-      <c r="C22" s="203" t="s">
+      <c r="C22" s="141" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="204" t="s">
+      <c r="D22" s="142" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="169"/>
-      <c r="B23" s="205" t="s">
+      <c r="B23" s="143" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="212">
+      <c r="C23" s="150">
         <v>-0.1</v>
       </c>
-      <c r="D23" s="213">
+      <c r="D23" s="151">
         <v>9.7999999999999997E-3</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="169"/>
-      <c r="B24" s="140" t="s">
+      <c r="B24" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="210">
+      <c r="C24" s="148">
         <v>5.8</v>
       </c>
-      <c r="D24" s="211">
+      <c r="D24" s="149">
         <v>1.12E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="169"/>
-    </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="76" t="s">
+      <c r="B26" s="207" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="76"/>
-      <c r="D26" s="76"/>
-      <c r="E26" s="76"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="76"/>
-      <c r="H26" s="76"/>
-      <c r="I26" s="76"/>
-      <c r="J26" s="76"/>
+      <c r="C26" s="207"/>
+      <c r="D26" s="207"/>
+      <c r="E26" s="207"/>
+      <c r="F26" s="207"/>
+      <c r="G26" s="207"/>
+      <c r="H26" s="207"/>
+      <c r="I26" s="207"/>
+      <c r="J26" s="207"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="169"/>
-      <c r="C28" s="170"/>
-      <c r="D28" s="182" t="s">
+      <c r="C28" s="116"/>
+      <c r="D28" s="128" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="182" t="s">
+      <c r="E28" s="128" t="s">
         <v>92</v>
       </c>
-      <c r="F28" s="182" t="s">
+      <c r="F28" s="128" t="s">
         <v>93</v>
       </c>
-      <c r="G28" s="182" t="s">
+      <c r="G28" s="128" t="s">
         <v>2</v>
       </c>
-      <c r="H28" s="182" t="s">
+      <c r="H28" s="128" t="s">
         <v>94</v>
       </c>
-      <c r="I28" s="186" t="s">
+      <c r="I28" s="130" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="169"/>
-      <c r="B29" s="196" t="s">
+      <c r="B29" s="208" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="197" t="s">
+      <c r="C29" s="137" t="s">
         <v>96</v>
       </c>
-      <c r="D29" s="191">
+      <c r="D29" s="134">
         <v>51.7</v>
       </c>
-      <c r="E29" s="192">
+      <c r="E29" s="135">
         <v>118.3</v>
       </c>
-      <c r="F29" s="192">
+      <c r="F29" s="135">
         <v>92.9</v>
       </c>
-      <c r="G29" s="192">
+      <c r="G29" s="135">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H29" s="192">
+      <c r="H29" s="135">
         <v>0.80200000000000005</v>
       </c>
-      <c r="I29" s="191">
+      <c r="I29" s="134">
         <v>73.400000000000006</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="169"/>
-      <c r="B30" s="199"/>
-      <c r="C30" s="200" t="s">
+      <c r="B30" s="209"/>
+      <c r="C30" s="138" t="s">
         <v>97</v>
       </c>
-      <c r="D30" s="141">
+      <c r="D30" s="88">
         <v>50.7</v>
       </c>
-      <c r="E30" s="176">
+      <c r="E30" s="122">
         <v>125.6</v>
       </c>
-      <c r="F30" s="176">
+      <c r="F30" s="122">
         <v>100.3</v>
       </c>
-      <c r="G30" s="176">
+      <c r="G30" s="122">
         <v>0.94120000000000004</v>
       </c>
-      <c r="H30" s="176">
+      <c r="H30" s="122">
         <v>0.76970000000000005</v>
       </c>
-      <c r="I30" s="141">
+      <c r="I30" s="88">
         <v>88.6</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="169"/>
-      <c r="B31" s="198" t="s">
+      <c r="B31" s="210" t="s">
         <v>14</v>
       </c>
-      <c r="C31" s="174" t="s">
+      <c r="C31" s="120" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="139">
+      <c r="D31" s="86">
         <v>50.2</v>
       </c>
-      <c r="E31" s="172">
+      <c r="E31" s="118">
         <v>123.7</v>
       </c>
-      <c r="F31" s="172">
+      <c r="F31" s="118">
         <v>100.3</v>
       </c>
-      <c r="G31" s="172">
+      <c r="G31" s="118">
         <v>0.94120000000000004</v>
       </c>
-      <c r="H31" s="172">
+      <c r="H31" s="118">
         <v>0.76890000000000003</v>
       </c>
-      <c r="I31" s="139">
+      <c r="I31" s="86">
         <v>79.099999999999994</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="169"/>
-      <c r="B32" s="199"/>
-      <c r="C32" s="200" t="s">
+      <c r="B32" s="209"/>
+      <c r="C32" s="138" t="s">
         <v>97</v>
       </c>
-      <c r="D32" s="141">
+      <c r="D32" s="88">
         <v>56.4</v>
       </c>
-      <c r="E32" s="176">
+      <c r="E32" s="122">
         <v>129.4</v>
       </c>
-      <c r="F32" s="176">
+      <c r="F32" s="122">
         <v>104.9</v>
       </c>
-      <c r="G32" s="176">
+      <c r="G32" s="122">
         <v>0.93569999999999998</v>
       </c>
-      <c r="H32" s="176">
+      <c r="H32" s="122">
         <v>0.74850000000000005</v>
       </c>
-      <c r="I32" s="141">
+      <c r="I32" s="88">
         <v>149.80000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C34" s="203" t="s">
+    <row r="34" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C34" s="141" t="s">
         <v>99</v>
       </c>
-      <c r="D34" s="202" t="s">
+      <c r="D34" s="140" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="169"/>
-      <c r="B35" s="201" t="s">
+    <row r="35" spans="2:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="139" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="214">
+      <c r="C35" s="152">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="D35" s="209">
+      <c r="D35" s="147">
         <v>8.3000000000000001E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="169"/>
-      <c r="B36" s="144" t="s">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="C36" s="210">
+      <c r="C36" s="148">
         <v>6.2</v>
       </c>
-      <c r="D36" s="211">
+      <c r="D36" s="149">
         <v>5.4999999999999997E-3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B14:J14"/>
     <mergeCell ref="B17:B18"/>
@@ -6864,6 +6845,8 @@
     <mergeCell ref="B26:J26"/>
     <mergeCell ref="B29:B30"/>
     <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6874,434 +6857,434 @@
   <dimension ref="B3:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="122" t="s">
+      <c r="B3" s="153" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="122"/>
-      <c r="D3" s="122"/>
-      <c r="E3" s="122"/>
-      <c r="F3" s="122"/>
+      <c r="C3" s="153"/>
+      <c r="D3" s="153"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="153"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="143"/>
-      <c r="C5" s="142" t="s">
+      <c r="B5" s="90"/>
+      <c r="C5" s="89" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="142" t="s">
+      <c r="D5" s="89" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="168" t="s">
+      <c r="B6" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="167">
+      <c r="C6" s="114">
         <v>50.7</v>
       </c>
-      <c r="D6" s="165">
+      <c r="D6" s="112">
         <v>0.94120000000000004</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="144" t="s">
+      <c r="B7" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="166">
+      <c r="C7" s="113">
         <v>56.4</v>
       </c>
-      <c r="D7" s="166">
+      <c r="D7" s="113">
         <v>0.93569999999999998</v>
       </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="122" t="s">
+      <c r="B25" s="153" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="122"/>
-      <c r="D25" s="122"/>
-      <c r="E25" s="122"/>
-      <c r="F25" s="122"/>
-      <c r="G25" s="122"/>
-      <c r="H25" s="122"/>
-      <c r="I25" s="122"/>
-      <c r="J25" s="122"/>
+      <c r="C25" s="153"/>
+      <c r="D25" s="153"/>
+      <c r="E25" s="153"/>
+      <c r="F25" s="153"/>
+      <c r="G25" s="153"/>
+      <c r="H25" s="153"/>
+      <c r="I25" s="153"/>
+      <c r="J25" s="153"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="123" t="s">
+      <c r="B27" s="154" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="124"/>
-      <c r="D27" s="124"/>
-      <c r="E27" s="124"/>
-      <c r="F27" s="124"/>
-      <c r="G27" s="124"/>
-      <c r="H27" s="124"/>
-      <c r="I27" s="124"/>
-      <c r="J27" s="125"/>
+      <c r="C27" s="155"/>
+      <c r="D27" s="155"/>
+      <c r="E27" s="155"/>
+      <c r="F27" s="155"/>
+      <c r="G27" s="155"/>
+      <c r="H27" s="155"/>
+      <c r="I27" s="155"/>
+      <c r="J27" s="156"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="127" t="s">
+      <c r="B28" s="77" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="127" t="s">
+      <c r="C28" s="77" t="s">
         <v>108</v>
       </c>
-      <c r="D28" s="127" t="s">
+      <c r="D28" s="77" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="127" t="s">
+      <c r="E28" s="77" t="s">
         <v>93</v>
       </c>
-      <c r="F28" s="127" t="s">
+      <c r="F28" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="G28" s="127" t="s">
+      <c r="G28" s="77" t="s">
         <v>105</v>
       </c>
-      <c r="H28" s="127" t="s">
+      <c r="H28" s="77" t="s">
         <v>112</v>
       </c>
-      <c r="I28" s="127" t="s">
+      <c r="I28" s="77" t="s">
         <v>106</v>
       </c>
-      <c r="J28" s="126" t="s">
+      <c r="J28" s="76" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="147" t="s">
+      <c r="B29" s="94" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="149" t="s">
+      <c r="C29" s="96" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="150">
+      <c r="D29" s="97">
         <v>74.385000000000005</v>
       </c>
-      <c r="E29" s="150">
+      <c r="E29" s="97">
         <v>140.24299999999999</v>
       </c>
-      <c r="F29" s="150">
+      <c r="F29" s="97">
         <v>0.88500000000000001</v>
       </c>
-      <c r="G29" s="150">
+      <c r="G29" s="97">
         <v>0.88490000000000002</v>
       </c>
-      <c r="H29" s="150">
+      <c r="H29" s="97">
         <v>46.482999999999997</v>
       </c>
-      <c r="I29" s="150">
+      <c r="I29" s="97">
         <v>22.6</v>
       </c>
-      <c r="J29" s="150">
+      <c r="J29" s="97">
         <v>-6.4500000000000002E-2</v>
       </c>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B30" s="128" t="s">
+      <c r="B30" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="148" t="s">
+      <c r="C30" s="95" t="s">
         <v>111</v>
       </c>
-      <c r="D30" s="151">
+      <c r="D30" s="98">
         <v>71.126999999999995</v>
       </c>
-      <c r="E30" s="151">
+      <c r="E30" s="98">
         <v>134.02699999999999</v>
       </c>
-      <c r="F30" s="151">
+      <c r="F30" s="98">
         <v>0.89500000000000002</v>
       </c>
-      <c r="G30" s="151">
+      <c r="G30" s="98">
         <v>0.89490000000000003</v>
       </c>
-      <c r="H30" s="151">
+      <c r="H30" s="98">
         <v>46.991999999999997</v>
       </c>
-      <c r="I30" s="151">
+      <c r="I30" s="98">
         <v>19.399999999999999</v>
       </c>
-      <c r="J30" s="151">
+      <c r="J30" s="98">
         <v>-5.45E-2</v>
       </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="128" t="s">
+      <c r="B31" s="78" t="s">
         <v>34</v>
       </c>
-      <c r="C31" s="130" t="s">
+      <c r="C31" s="80" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="152">
+      <c r="D31" s="99">
         <v>71.126999999999995</v>
       </c>
-      <c r="E31" s="152">
+      <c r="E31" s="99">
         <v>134.02699999999999</v>
       </c>
-      <c r="F31" s="152">
+      <c r="F31" s="99">
         <v>0.89500000000000002</v>
       </c>
-      <c r="G31" s="152">
+      <c r="G31" s="99">
         <v>0.89490000000000003</v>
       </c>
-      <c r="H31" s="152">
+      <c r="H31" s="99">
         <v>46.822000000000003</v>
       </c>
-      <c r="I31" s="152">
+      <c r="I31" s="99">
         <v>19.399999999999999</v>
       </c>
-      <c r="J31" s="153">
+      <c r="J31" s="100">
         <v>-5.45E-2</v>
       </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="128" t="s">
+      <c r="B32" s="78" t="s">
         <v>113</v>
       </c>
-      <c r="C32" s="148" t="s">
+      <c r="C32" s="95" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="151">
+      <c r="D32" s="98">
         <v>71.126999999999995</v>
       </c>
-      <c r="E32" s="151">
+      <c r="E32" s="98">
         <v>134.02699999999999</v>
       </c>
-      <c r="F32" s="151">
+      <c r="F32" s="98">
         <v>0.89500000000000002</v>
       </c>
-      <c r="G32" s="151">
+      <c r="G32" s="98">
         <v>0.89490000000000003</v>
       </c>
-      <c r="H32" s="151">
+      <c r="H32" s="98">
         <v>46.822000000000003</v>
       </c>
-      <c r="I32" s="151">
+      <c r="I32" s="98">
         <v>19.399999999999999</v>
       </c>
-      <c r="J32" s="151">
+      <c r="J32" s="98">
         <v>-5.45E-2</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="129" t="s">
+      <c r="B33" s="79" t="s">
         <v>114</v>
       </c>
-      <c r="C33" s="131">
+      <c r="C33" s="81">
         <v>3925</v>
       </c>
-      <c r="D33" s="154">
+      <c r="D33" s="101">
         <v>154.19999999999999</v>
       </c>
-      <c r="E33" s="154">
+      <c r="E33" s="101">
         <v>197.601</v>
       </c>
-      <c r="F33" s="154">
+      <c r="F33" s="101">
         <v>0.65529999999999999</v>
       </c>
-      <c r="G33" s="154">
+      <c r="G33" s="101">
         <v>0.65449999999999997</v>
       </c>
-      <c r="H33" s="154">
+      <c r="H33" s="101">
         <v>46.822000000000003</v>
       </c>
-      <c r="I33" s="154" t="s">
+      <c r="I33" s="101" t="s">
         <v>115</v>
       </c>
-      <c r="J33" s="155" t="s">
+      <c r="J33" s="102" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="132" t="s">
+      <c r="B35" s="157" t="s">
         <v>116</v>
       </c>
-      <c r="C35" s="133"/>
-      <c r="D35" s="133"/>
-      <c r="E35" s="133"/>
-      <c r="F35" s="133"/>
-      <c r="G35" s="133"/>
-      <c r="H35" s="133"/>
-      <c r="I35" s="133"/>
-      <c r="J35" s="134"/>
+      <c r="C35" s="158"/>
+      <c r="D35" s="158"/>
+      <c r="E35" s="158"/>
+      <c r="F35" s="158"/>
+      <c r="G35" s="158"/>
+      <c r="H35" s="158"/>
+      <c r="I35" s="158"/>
+      <c r="J35" s="159"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="137" t="s">
+      <c r="B36" s="84" t="s">
         <v>109</v>
       </c>
-      <c r="C36" s="137" t="s">
+      <c r="C36" s="84" t="s">
         <v>108</v>
       </c>
-      <c r="D36" s="137" t="s">
+      <c r="D36" s="84" t="s">
         <v>91</v>
       </c>
-      <c r="E36" s="137" t="s">
+      <c r="E36" s="84" t="s">
         <v>93</v>
       </c>
-      <c r="F36" s="135" t="s">
+      <c r="F36" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="G36" s="137" t="s">
+      <c r="G36" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="H36" s="135" t="s">
+      <c r="H36" s="82" t="s">
         <v>112</v>
       </c>
-      <c r="I36" s="137" t="s">
+      <c r="I36" s="84" t="s">
         <v>106</v>
       </c>
-      <c r="J36" s="136" t="s">
+      <c r="J36" s="83" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="145" t="s">
+      <c r="B37" s="92" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="156" t="s">
+      <c r="C37" s="103" t="s">
         <v>111</v>
       </c>
-      <c r="D37" s="156">
+      <c r="D37" s="103">
         <v>221.876</v>
       </c>
-      <c r="E37" s="156">
+      <c r="E37" s="103">
         <v>397.423</v>
       </c>
-      <c r="F37" s="157">
+      <c r="F37" s="104">
         <v>7.6499999999999999E-2</v>
       </c>
-      <c r="G37" s="156">
+      <c r="G37" s="103">
         <v>7.5800000000000006E-2</v>
       </c>
-      <c r="H37" s="157">
+      <c r="H37" s="104">
         <v>31.99</v>
       </c>
-      <c r="I37" s="156">
+      <c r="I37" s="103">
         <v>173.8</v>
       </c>
-      <c r="J37" s="158">
+      <c r="J37" s="105">
         <v>-0.86209999999999998</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="146" t="s">
+      <c r="B38" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="159" t="s">
+      <c r="C38" s="106" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="159">
+      <c r="D38" s="106">
         <v>259.61200000000002</v>
       </c>
-      <c r="E38" s="159">
+      <c r="E38" s="106">
         <v>328.69499999999999</v>
       </c>
-      <c r="F38" s="159">
+      <c r="F38" s="106">
         <v>0.36830000000000002</v>
       </c>
-      <c r="G38" s="159">
+      <c r="G38" s="106">
         <v>0.36780000000000002</v>
       </c>
-      <c r="H38" s="159">
+      <c r="H38" s="106">
         <v>32.792000000000002</v>
       </c>
-      <c r="I38" s="159">
+      <c r="I38" s="106">
         <v>211.5</v>
       </c>
-      <c r="J38" s="159">
+      <c r="J38" s="106">
         <v>-0.57030000000000003</v>
       </c>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="146" t="s">
+      <c r="B39" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="160" t="s">
+      <c r="C39" s="107" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="160">
+      <c r="D39" s="107">
         <v>259.61200000000002</v>
       </c>
-      <c r="E39" s="160">
+      <c r="E39" s="107">
         <v>328.69499999999999</v>
       </c>
-      <c r="F39" s="161">
+      <c r="F39" s="108">
         <v>0.36830000000000002</v>
       </c>
-      <c r="G39" s="160">
+      <c r="G39" s="107">
         <v>0.36780000000000002</v>
       </c>
-      <c r="H39" s="160">
+      <c r="H39" s="107">
         <v>32.398000000000003</v>
       </c>
-      <c r="I39" s="160">
+      <c r="I39" s="107">
         <v>211.5</v>
       </c>
-      <c r="J39" s="160">
+      <c r="J39" s="107">
         <v>-0.57030000000000003</v>
       </c>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="146" t="s">
+      <c r="B40" s="93" t="s">
         <v>113</v>
       </c>
-      <c r="C40" s="159" t="s">
+      <c r="C40" s="106" t="s">
         <v>111</v>
       </c>
-      <c r="D40" s="159">
+      <c r="D40" s="106">
         <v>259.61200000000002</v>
       </c>
-      <c r="E40" s="159">
+      <c r="E40" s="106">
         <v>328.69499999999999</v>
       </c>
-      <c r="F40" s="159">
+      <c r="F40" s="106">
         <v>0.36830000000000002</v>
       </c>
-      <c r="G40" s="159">
+      <c r="G40" s="106">
         <v>0.36780000000000002</v>
       </c>
-      <c r="H40" s="159">
+      <c r="H40" s="106">
         <v>32.398000000000003</v>
       </c>
-      <c r="I40" s="159">
+      <c r="I40" s="106">
         <v>211.5</v>
       </c>
-      <c r="J40" s="159">
+      <c r="J40" s="106">
         <v>-0.57030000000000003</v>
       </c>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B41" s="138" t="s">
+      <c r="B41" s="85" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="162">
+      <c r="C41" s="109">
         <v>3935</v>
       </c>
-      <c r="D41" s="162">
+      <c r="D41" s="109">
         <v>396.416</v>
       </c>
-      <c r="E41" s="162">
+      <c r="E41" s="109">
         <v>476.995</v>
       </c>
-      <c r="F41" s="163">
+      <c r="F41" s="110">
         <v>-1.0088999999999999</v>
       </c>
-      <c r="G41" s="162">
+      <c r="G41" s="109">
         <v>-1.0129999999999999</v>
       </c>
-      <c r="H41" s="163">
+      <c r="H41" s="110">
         <v>32.398000000000003</v>
       </c>
-      <c r="I41" s="162" t="s">
+      <c r="I41" s="109" t="s">
         <v>115</v>
       </c>
-      <c r="J41" s="164" t="s">
+      <c r="J41" s="111" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>